<commit_message>
add: PDFs da matriz comunitária e planilha de cortes atualizada
</commit_message>
<xml_diff>
--- a/revista/modelo/planilhas importantes/Cortes dos Padrões por Etapa e Parceiro.xlsx
+++ b/revista/modelo/planilhas importantes/Cortes dos Padrões por Etapa e Parceiro.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="2EF - LP" sheetId="1" state="visible" r:id="rId3"/>
@@ -390,104 +390,108 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -869,388 +873,388 @@
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="6" t="s">
+      <c r="C3" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="C4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="C5" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="C7" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8"/>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="9"/>
+      <c r="B8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="6" t="s">
+      <c r="C8" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
-      <c r="B9" s="7" t="s">
+      <c r="A9" s="9"/>
+      <c r="B9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="C9" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8"/>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="6" t="s">
+      <c r="C10" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="9"/>
+      <c r="B11" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="C11" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8"/>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="C12" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8"/>
-      <c r="B13" s="7" t="s">
+      <c r="A13" s="9"/>
+      <c r="B13" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="C13" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8"/>
-      <c r="B14" s="7" t="s">
+      <c r="A14" s="9"/>
+      <c r="B14" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D14" s="6" t="s">
+      <c r="C14" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8"/>
-      <c r="B15" s="7" t="s">
+      <c r="A15" s="9"/>
+      <c r="B15" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="6" t="s">
+      <c r="C15" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8"/>
-      <c r="B16" s="7" t="s">
+      <c r="A16" s="9"/>
+      <c r="B16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="6" t="s">
+      <c r="C16" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8"/>
-      <c r="B17" s="7" t="s">
+      <c r="A17" s="9"/>
+      <c r="B17" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="6" t="s">
+      <c r="C17" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8"/>
-      <c r="B18" s="7" t="s">
+      <c r="A18" s="9"/>
+      <c r="B18" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="6" t="s">
+      <c r="C18" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8"/>
-      <c r="B19" s="7" t="s">
+      <c r="A19" s="9"/>
+      <c r="B19" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="6" t="s">
+      <c r="C19" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8"/>
-      <c r="B20" s="7" t="s">
+      <c r="A20" s="9"/>
+      <c r="B20" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="6" t="s">
+      <c r="C20" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8"/>
-      <c r="B21" s="7" t="s">
+      <c r="A21" s="9"/>
+      <c r="B21" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="C21" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8"/>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="9"/>
+      <c r="B22" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="6" t="s">
+      <c r="C22" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8"/>
-      <c r="B23" s="7" t="s">
+      <c r="A23" s="9"/>
+      <c r="B23" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="6" t="s">
+      <c r="C23" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8"/>
-      <c r="B24" s="7" t="s">
+      <c r="A24" s="9"/>
+      <c r="B24" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="6" t="s">
+      <c r="C24" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8"/>
-      <c r="B25" s="7" t="s">
+      <c r="A25" s="9"/>
+      <c r="B25" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="6" t="s">
+      <c r="C25" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="6" t="s">
+      <c r="C27" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8"/>
-      <c r="B28" s="7" t="s">
+      <c r="A28" s="9"/>
+      <c r="B28" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C28" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="6" t="s">
+      <c r="C28" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8"/>
-      <c r="B29" s="7" t="s">
+      <c r="A29" s="9"/>
+      <c r="B29" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C29" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="6" t="s">
+      <c r="C29" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="4" t="s">
+      <c r="C30" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="5" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1283,385 +1287,385 @@
   <dimension ref="A1:D30"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="6" t="s">
+      <c r="C2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="6" t="s">
+      <c r="C4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9"/>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="10"/>
+      <c r="B6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="C6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9"/>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="10"/>
+      <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="C7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9"/>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="10"/>
+      <c r="B8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="C8" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9"/>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="10"/>
+      <c r="B9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="4" t="s">
+      <c r="C9" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9"/>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="10"/>
+      <c r="B10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C10" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="10"/>
+      <c r="B11" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="C11" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="10"/>
+      <c r="B12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="10"/>
+      <c r="B13" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="C13" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="10"/>
+      <c r="B14" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="C14" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="10"/>
+      <c r="B15" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="4" t="s">
+      <c r="C15" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9"/>
-      <c r="B16" s="5" t="s">
+      <c r="A16" s="10"/>
+      <c r="B16" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="C16" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9"/>
-      <c r="B17" s="5" t="s">
+      <c r="A17" s="10"/>
+      <c r="B17" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="C17" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9"/>
-      <c r="B18" s="5" t="s">
+      <c r="A18" s="10"/>
+      <c r="B18" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9"/>
-      <c r="B19" s="5" t="s">
+      <c r="A19" s="10"/>
+      <c r="B19" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="C19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="5" t="s">
+      <c r="A20" s="10"/>
+      <c r="B20" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="4" t="s">
+      <c r="C20" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9"/>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="10"/>
+      <c r="B21" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="C21" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9"/>
-      <c r="B22" s="5" t="s">
+      <c r="A22" s="10"/>
+      <c r="B22" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="C22" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="9"/>
-      <c r="B23" s="5" t="s">
+      <c r="A23" s="10"/>
+      <c r="B23" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="C23" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B24" s="7" t="s">
+      <c r="A24" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C24" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="6" t="s">
+      <c r="C24" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8"/>
-      <c r="B25" s="7" t="s">
+      <c r="A25" s="9"/>
+      <c r="B25" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="6" t="s">
+      <c r="C25" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="4" t="s">
+      <c r="C26" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="n">
+      <c r="A27" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="6" t="s">
+      <c r="C27" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8"/>
-      <c r="B28" s="7" t="s">
+      <c r="A28" s="9"/>
+      <c r="B28" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C28" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="6" t="s">
+      <c r="C28" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8"/>
-      <c r="B29" s="7" t="s">
+      <c r="A29" s="9"/>
+      <c r="B29" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C29" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="6" t="s">
+      <c r="C29" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8"/>
-      <c r="B30" s="7" t="s">
+      <c r="A30" s="9"/>
+      <c r="B30" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C30" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="6" t="s">
+      <c r="C30" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1695,296 +1699,296 @@
   <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="17.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="17"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="4" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="n">
+      <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" s="12" t="s">
+      <c r="C2" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D3" s="13" t="s">
+      <c r="C3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="n">
+      <c r="A4" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="12" t="s">
+      <c r="C4" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14"/>
-      <c r="B5" s="11" t="s">
+      <c r="A5" s="15"/>
+      <c r="B5" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="12" t="s">
+      <c r="C5" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="13" t="s">
+      <c r="C6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9"/>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="10"/>
+      <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="13" t="s">
+      <c r="C7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9"/>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="10"/>
+      <c r="B8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="13" t="s">
+      <c r="C8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9"/>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="10"/>
+      <c r="B9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" s="13" t="s">
+      <c r="C9" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9"/>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="10"/>
+      <c r="B10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="13" t="s">
+      <c r="C10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="10"/>
+      <c r="B11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" s="13" t="s">
+      <c r="C11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="10"/>
+      <c r="B12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="13" t="s">
+      <c r="C12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="10"/>
+      <c r="B13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D13" s="13" t="s">
+      <c r="C13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="10"/>
+      <c r="B14" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" s="13" t="s">
+      <c r="C14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="10"/>
+      <c r="B15" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="13" t="s">
+      <c r="C15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9"/>
-      <c r="B16" s="5" t="s">
+      <c r="A16" s="10"/>
+      <c r="B16" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="13" t="s">
+      <c r="C16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9"/>
-      <c r="B17" s="5" t="s">
+      <c r="A17" s="10"/>
+      <c r="B17" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="13" t="s">
+      <c r="C17" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9"/>
-      <c r="B18" s="5" t="s">
+      <c r="A18" s="10"/>
+      <c r="B18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" s="13" t="s">
+      <c r="C18" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9"/>
-      <c r="B19" s="5" t="s">
+      <c r="A19" s="10"/>
+      <c r="B19" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="13" t="s">
+      <c r="C19" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="5" t="s">
+      <c r="A20" s="10"/>
+      <c r="B20" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="13" t="s">
+      <c r="C20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9"/>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="10"/>
+      <c r="B21" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D21" s="13" t="s">
+      <c r="C21" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9"/>
-      <c r="B22" s="5" t="s">
+      <c r="A22" s="10"/>
+      <c r="B22" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" s="13" t="s">
+      <c r="C22" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="14" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="B23" s="11" t="s">
+      <c r="A23" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" s="12" t="s">
+      <c r="C23" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="13" t="s">
         <v>53</v>
       </c>
     </row>
@@ -2018,295 +2022,297 @@
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="15" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="16" width="18.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="n">
+      <c r="A2" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" s="18" t="s">
+      <c r="C2" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="19" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D3" s="19" t="s">
+      <c r="C3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="20" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="n">
+      <c r="A4" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="18" t="s">
+      <c r="C4" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="19" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20"/>
-      <c r="B5" s="17" t="s">
+      <c r="A5" s="21"/>
+      <c r="B5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="C5" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="19" t="s">
+      <c r="C6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9"/>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="10"/>
+      <c r="B7" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="19" t="s">
+      <c r="C7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9"/>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="10"/>
+      <c r="B8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D8" s="19" t="s">
+      <c r="C8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9"/>
-      <c r="B9" s="5" t="s">
+      <c r="A9" s="10"/>
+      <c r="B9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" s="19" t="s">
+      <c r="C9" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9"/>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="10"/>
+      <c r="B10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10" s="19" t="s">
+      <c r="C10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="10"/>
+      <c r="B11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D11" s="19" t="s">
+      <c r="C11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="10"/>
+      <c r="B12" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D12" s="19" t="s">
+      <c r="C12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="10"/>
+      <c r="B13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D13" s="19" t="s">
+      <c r="C13" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="10"/>
+      <c r="B14" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" s="19" t="s">
+      <c r="C14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9"/>
-      <c r="B15" s="5" t="s">
+      <c r="A15" s="10"/>
+      <c r="B15" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="19" t="s">
+      <c r="C15" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9"/>
-      <c r="B16" s="5" t="s">
+      <c r="A16" s="10"/>
+      <c r="B16" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="19" t="s">
+      <c r="C16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9"/>
-      <c r="B17" s="5" t="s">
+      <c r="A17" s="10"/>
+      <c r="B17" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D17" s="19" t="s">
+      <c r="C17" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9"/>
-      <c r="B18" s="5" t="s">
+      <c r="A18" s="10"/>
+      <c r="B18" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" s="19" t="s">
+      <c r="C18" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9"/>
-      <c r="B19" s="5" t="s">
+      <c r="A19" s="10"/>
+      <c r="B19" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" s="19" t="s">
+      <c r="C19" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="5" t="s">
+      <c r="A20" s="10"/>
+      <c r="B20" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D20" s="19" t="s">
+      <c r="C20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9"/>
-      <c r="B21" s="5" t="s">
+      <c r="A21" s="10"/>
+      <c r="B21" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D21" s="19" t="s">
+      <c r="C21" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" s="20" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B22" s="17" t="s">
+      <c r="A22" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" s="18" t="s">
+      <c r="C22" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="19" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4"/>
-      <c r="B23" s="5" t="s">
+      <c r="A23" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" s="19" t="s">
+      <c r="C23" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="20" t="s">
         <v>57</v>
       </c>
     </row>
@@ -2333,285 +2339,285 @@
   <dimension ref="A1:E20"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="2" width="18.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3"/>
+      <c r="E1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="n">
+      <c r="A2" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="22" t="s">
+      <c r="C2" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E2" s="15"/>
+      <c r="E2" s="16"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="23" t="n">
+      <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="23" t="s">
+      <c r="C3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="15"/>
+      <c r="E3" s="16"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="n">
+      <c r="A4" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="22" t="s">
+      <c r="C4" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="E4" s="15"/>
+      <c r="E4" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="23" t="s">
+      <c r="C5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="15"/>
+      <c r="E5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9"/>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="10"/>
+      <c r="B6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="23" t="s">
+      <c r="C6" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="E6" s="15"/>
+      <c r="E6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9"/>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="10"/>
+      <c r="B7" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" s="23" t="s">
+      <c r="C7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="15"/>
+      <c r="E7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="22" t="s">
+      <c r="C8" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E8" s="15"/>
+      <c r="E8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
-      <c r="B9" s="7" t="s">
+      <c r="A9" s="9"/>
+      <c r="B9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="22" t="s">
+      <c r="C9" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="15"/>
+      <c r="E9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8"/>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="22" t="s">
+      <c r="C10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="15"/>
+      <c r="E10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="9"/>
+      <c r="B11" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="22" t="s">
+      <c r="C11" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E11" s="15"/>
+      <c r="E11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8"/>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="22" t="s">
+      <c r="C12" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E12" s="15"/>
+      <c r="E12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8"/>
-      <c r="B13" s="7" t="s">
+      <c r="A13" s="9"/>
+      <c r="B13" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D13" s="22" t="s">
+      <c r="C13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E13" s="15"/>
+      <c r="E13" s="16"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8"/>
-      <c r="B14" s="7" t="s">
+      <c r="A14" s="9"/>
+      <c r="B14" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="22" t="s">
+      <c r="C14" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="15"/>
+      <c r="E14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8"/>
-      <c r="B15" s="7" t="s">
+      <c r="A15" s="9"/>
+      <c r="B15" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D15" s="22" t="s">
+      <c r="C15" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E15" s="15"/>
+      <c r="E15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8"/>
-      <c r="B16" s="7" t="s">
+      <c r="A16" s="9"/>
+      <c r="B16" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="22" t="s">
+      <c r="C16" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="15"/>
+      <c r="E16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8"/>
-      <c r="B17" s="7" t="s">
+      <c r="A17" s="9"/>
+      <c r="B17" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="22" t="s">
+      <c r="C17" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E17" s="15"/>
+      <c r="E17" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8"/>
-      <c r="B18" s="7" t="s">
+      <c r="A18" s="9"/>
+      <c r="B18" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="22" t="s">
+      <c r="C18" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="E18" s="15"/>
+      <c r="E18" s="16"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="n">
+      <c r="A19" s="24" t="n">
         <v>6</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="23" t="s">
+      <c r="C19" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="E19" s="15"/>
+      <c r="E19" s="16"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22" t="n">
+      <c r="A20" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="22" t="s">
+      <c r="C20" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E20" s="15"/>
+      <c r="E20" s="16"/>
     </row>
   </sheetData>
   <autoFilter ref="B1:E1">
@@ -2642,263 +2648,263 @@
   <dimension ref="A1:D20"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="10.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="18.42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D2" s="22" t="s">
+      <c r="C2" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="23" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="23" t="s">
+      <c r="C3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="24" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" s="22" t="s">
+      <c r="C4" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="23" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" s="23" t="s">
+      <c r="C5" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="24" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9"/>
-      <c r="B6" s="5" t="s">
+      <c r="A6" s="10"/>
+      <c r="B6" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" s="23" t="s">
+      <c r="C6" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D6" s="24" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9"/>
-      <c r="B7" s="5" t="s">
+      <c r="A7" s="10"/>
+      <c r="B7" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" s="23" t="s">
+      <c r="C7" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="24" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" s="22" t="s">
+      <c r="C8" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8"/>
-      <c r="B9" s="7" t="s">
+      <c r="A9" s="9"/>
+      <c r="B9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="22" t="s">
+      <c r="C9" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8"/>
-      <c r="B10" s="7" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" s="22" t="s">
+      <c r="C10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8"/>
-      <c r="B11" s="7" t="s">
+      <c r="A11" s="9"/>
+      <c r="B11" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="22" t="s">
+      <c r="C11" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8"/>
-      <c r="B12" s="7" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="22" t="s">
+      <c r="C12" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D12" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8"/>
-      <c r="B13" s="7" t="s">
+      <c r="A13" s="9"/>
+      <c r="B13" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D13" s="22" t="s">
+      <c r="C13" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8"/>
-      <c r="B14" s="7" t="s">
+      <c r="A14" s="9"/>
+      <c r="B14" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" s="22" t="s">
+      <c r="C14" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8"/>
-      <c r="B15" s="7" t="s">
+      <c r="A15" s="9"/>
+      <c r="B15" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D15" s="22" t="s">
+      <c r="C15" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8"/>
-      <c r="B16" s="7" t="s">
+      <c r="A16" s="9"/>
+      <c r="B16" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="22" t="s">
+      <c r="C16" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8"/>
-      <c r="B17" s="7" t="s">
+      <c r="A17" s="9"/>
+      <c r="B17" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D17" s="22" t="s">
+      <c r="C17" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8"/>
-      <c r="B18" s="7" t="s">
+      <c r="A18" s="9"/>
+      <c r="B18" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D18" s="22" t="s">
+      <c r="C18" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="23" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8"/>
-      <c r="B19" s="7" t="s">
+      <c r="A19" s="9"/>
+      <c r="B19" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="22" t="s">
+      <c r="C19" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="23" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="23" t="s">
+      <c r="C20" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="24" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2931,205 +2937,205 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="15" width="18.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="16" width="18.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="n">
+      <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="D2" s="24" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="24" t="n">
+      <c r="A3" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="D3" s="25" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="n">
+      <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="24" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="n">
+      <c r="A5" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="25" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20"/>
-      <c r="B6" s="17" t="s">
+      <c r="A6" s="21"/>
+      <c r="B6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="25" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20"/>
-      <c r="B7" s="17" t="s">
+      <c r="A7" s="21"/>
+      <c r="B7" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="25" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D8" s="23" t="s">
+      <c r="D8" s="24" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="n">
+      <c r="A9" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="25" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20"/>
-      <c r="B10" s="17" t="s">
+      <c r="A10" s="21"/>
+      <c r="B10" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="25" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20"/>
-      <c r="B11" s="17" t="s">
+      <c r="A11" s="21"/>
+      <c r="B11" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="D11" s="25" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20"/>
-      <c r="B12" s="17" t="s">
+      <c r="A12" s="21"/>
+      <c r="B12" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="25" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20"/>
-      <c r="B13" s="17" t="s">
+      <c r="A13" s="21"/>
+      <c r="B13" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="24" t="s">
+      <c r="D13" s="25" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20"/>
-      <c r="B14" s="17" t="s">
+      <c r="A14" s="21"/>
+      <c r="B14" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D14" s="24" t="s">
+      <c r="D14" s="25" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="n">
+      <c r="A15" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="24" t="s">
         <v>74</v>
       </c>
     </row>
@@ -3165,204 +3171,204 @@
   <dimension ref="A1:D15"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="15" width="18.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="16" width="18.42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="n">
+      <c r="A2" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="25" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="24" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="n">
+      <c r="A4" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20"/>
-      <c r="B5" s="17" t="s">
+      <c r="A5" s="21"/>
+      <c r="B5" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="D5" s="25" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20"/>
-      <c r="B6" s="17" t="s">
+      <c r="A6" s="21"/>
+      <c r="B6" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="25" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="24" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="17" t="s">
+      <c r="A8" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="25" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="24" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9"/>
-      <c r="B10" s="5" t="s">
+      <c r="A10" s="10"/>
+      <c r="B10" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="24" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="10"/>
+      <c r="B11" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="24" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="5" t="s">
+      <c r="A12" s="10"/>
+      <c r="B12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="24" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9"/>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="10"/>
+      <c r="B13" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="24" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="5" t="s">
+      <c r="A14" s="10"/>
+      <c r="B14" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="24" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="16" t="n">
+      <c r="A15" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="24" t="s">
+      <c r="D15" s="25" t="s">
         <v>77</v>
       </c>
     </row>

</xml_diff>